<commit_message>
all components placed on pcb
just need to route it now
</commit_message>
<xml_diff>
--- a/MM_26 Bill of Parts.xlsx
+++ b/MM_26 Bill of Parts.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\james\Documents\Github\Micromouse-2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBDC6FF0-58E3-436B-BF66-F352A6D162A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B10286D8-F4A4-491D-810C-E0B2C1B83B7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{C0469B51-F70B-4F72-8A5A-A226DBC3104A}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="60">
   <si>
     <t>Part</t>
   </si>
@@ -210,6 +210,12 @@
   </si>
   <si>
     <t>https://www.pololu.com/product/2703</t>
+  </si>
+  <si>
+    <t>Motor Bracket</t>
+  </si>
+  <si>
+    <t>https://www.pololu.com/category/161/brackets-for-micro-metal-gearmotors</t>
   </si>
 </sst>
 </file>
@@ -622,7 +628,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D335EDAF-01BC-43D0-BDFE-27332DC556ED}">
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="19.08984375" bestFit="1" customWidth="1"/>
@@ -1026,6 +1032,23 @@
         <v>57</v>
       </c>
     </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>58</v>
+      </c>
+      <c r="B17">
+        <v>1</v>
+      </c>
+      <c r="D17" s="1">
+        <v>4.95</v>
+      </c>
+      <c r="E17">
+        <v>1089</v>
+      </c>
+      <c r="F17" t="s">
+        <v>59</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B15:H15"/>

</xml_diff>

<commit_message>
cut the thing in half
forgot to upload this earlier
</commit_message>
<xml_diff>
--- a/MM_26 Bill of Parts.xlsx
+++ b/MM_26 Bill of Parts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\james\Documents\Github\Micromouse-2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B10286D8-F4A4-491D-810C-E0B2C1B83B7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34A7F675-2F06-44A7-9AF4-E689DB5E8125}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{C0469B51-F70B-4F72-8A5A-A226DBC3104A}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="80">
   <si>
     <t>Part</t>
   </si>
@@ -164,12 +164,6 @@
     <t>Slide Switch</t>
   </si>
   <si>
-    <t>563-1314-1-ND</t>
-  </si>
-  <si>
-    <t>https://www.digikey.com/en/products/detail/nidec-components-corporation/CL-SB-12A-01T/3507814</t>
-  </si>
-  <si>
     <t>Switch</t>
   </si>
   <si>
@@ -216,6 +210,72 @@
   </si>
   <si>
     <t>https://www.pololu.com/category/161/brackets-for-micro-metal-gearmotors</t>
+  </si>
+  <si>
+    <t>Resistor</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/yageo/RC0805JR-0710KL/728241</t>
+  </si>
+  <si>
+    <t>100nF</t>
+  </si>
+  <si>
+    <t>4.7uF</t>
+  </si>
+  <si>
+    <t>10uF</t>
+  </si>
+  <si>
+    <t>22uF</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/kemet/C0805C104K5RACTU/411169</t>
+  </si>
+  <si>
+    <t>399-C0805C104K5RACTUCT-ND</t>
+  </si>
+  <si>
+    <t>1276-1244-1-ND</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/samsung-electro-mechanics/CL21A475KAQNNNE/3886902</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/samsung-electro-mechanics/CL21B106KOQNNNE/3888530</t>
+  </si>
+  <si>
+    <t>1276-2872-1-ND</t>
+  </si>
+  <si>
+    <t>1276-CL21A226MAYNNNECT-ND</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/samsung-electro-mechanics/CL21A226MAYNNNE/10479857</t>
+  </si>
+  <si>
+    <t>IDC Cable Header</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/cnc-tech/3220-20-0100-00/3883663</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/samtec-inc/FFSD-10-D-02-00-01-N/1106582</t>
+  </si>
+  <si>
+    <t>Cable Long</t>
+  </si>
+  <si>
+    <t>Cable Short</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/samtec-inc/FFSD-10-D-03-00-01-N/2651117</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/e-switch/EG1213/101735</t>
+  </si>
+  <si>
+    <t>EG1906-ND</t>
   </si>
 </sst>
 </file>
@@ -628,7 +688,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D335EDAF-01BC-43D0-BDFE-27332DC556ED}">
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="19.08984375" bestFit="1" customWidth="1"/>
@@ -775,7 +835,7 @@
         <v>8.7899999999999991</v>
       </c>
       <c r="I5" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.35">
@@ -864,7 +924,7 @@
         <v>25</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D9" s="7"/>
       <c r="E9" s="7"/>
@@ -872,7 +932,7 @@
       <c r="G9" s="7"/>
       <c r="H9" s="7"/>
       <c r="I9" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.35">
@@ -952,28 +1012,31 @@
         <v>41</v>
       </c>
       <c r="B13">
+        <v>2</v>
+      </c>
+      <c r="C13">
         <v>1</v>
       </c>
       <c r="D13" s="1">
-        <v>1.1000000000000001</v>
+        <v>0.72</v>
       </c>
       <c r="E13" t="s">
-        <v>42</v>
+        <v>79</v>
       </c>
       <c r="F13" s="2" t="str">
         <f t="shared" si="1"/>
-        <v>https://www.digikey.com/en/products/detail/nidec-components-corporation/CL-SB-12A-01T/3507814</v>
+        <v>https://www.digikey.com/en/products/detail/e-switch/EG1213/101735</v>
       </c>
       <c r="G13" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="I13" t="s">
-        <v>43</v>
+        <v>78</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B14">
         <v>2</v>
@@ -982,25 +1045,25 @@
         <v>0.67</v>
       </c>
       <c r="E14" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="F14" s="2" t="str">
         <f t="shared" si="1"/>
         <v>www.digikey.com/en/products/detail/jst-sales-america-inc/BM06B-SRSS-TB/926698</v>
       </c>
       <c r="G14" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="I14" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
+        <v>47</v>
+      </c>
+      <c r="B15" s="7" t="s">
         <v>49</v>
-      </c>
-      <c r="B15" s="7" t="s">
-        <v>51</v>
       </c>
       <c r="C15" s="7"/>
       <c r="D15" s="7"/>
@@ -1009,12 +1072,12 @@
       <c r="G15" s="7"/>
       <c r="H15" s="7"/>
       <c r="I15" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B16">
         <v>5</v>
@@ -1026,15 +1089,15 @@
         <v>2703</v>
       </c>
       <c r="G16" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="I16" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B17">
         <v>1</v>
@@ -1046,7 +1109,92 @@
         <v>1089</v>
       </c>
       <c r="F17" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>58</v>
+      </c>
+      <c r="B18">
+        <v>1</v>
+      </c>
+      <c r="C18">
+        <v>9</v>
+      </c>
+      <c r="D18" s="1">
+        <v>8.9999999999999993E-3</v>
+      </c>
+      <c r="F18" t="s">
         <v>59</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>60</v>
+      </c>
+      <c r="E19" t="s">
+        <v>65</v>
+      </c>
+      <c r="F19" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>61</v>
+      </c>
+      <c r="E20" t="s">
+        <v>66</v>
+      </c>
+      <c r="F20" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>62</v>
+      </c>
+      <c r="E21" t="s">
+        <v>69</v>
+      </c>
+      <c r="F21" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>63</v>
+      </c>
+      <c r="E22" t="s">
+        <v>70</v>
+      </c>
+      <c r="F22" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>72</v>
+      </c>
+      <c r="F23" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>76</v>
+      </c>
+      <c r="F24" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>75</v>
+      </c>
+      <c r="F25" t="s">
+        <v>77</v>
       </c>
     </row>
   </sheetData>

</xml_diff>